<commit_message>
Add Cinderella (1950) to Tier 2
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="484">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1462,6 +1462,12 @@
   </si>
   <si>
     <t xml:space="preserve">genre gate trivial -- real curse magic (Maleficent's 100-years'-sleep curse is the entire plot engine), a fairy-granted 'gift' downgrade, three fairy godmothers with real protective magic, and a literal dragon transformation in the climax. Structural Despair (0), Limited Heroism (0), Moral Cynicism (0), and Redemption Difficulty (0) since the curse is fully and permanently broken, the kingdom fully restored, and no character arc centers on atonement for real wrongdoing. Structural Corruption (0): dug further into Maleficent's actual dominion for this entry specifically -- she operates from her own separate domain (the Forbidden Mountains, her own castle, her own goon army) as an external aggressor against a neighboring legitimate kingdom, but she never rules over or oppresses King Stefan's own subjects, so this doesn't reach the bar this catalog has set for institutional tyranny (contrast The Wizard of Oz and Alice in Wonderland (2010-2016), both SC=2, where the Wicked Witch/Red Queen actually enslave or execute their own subject populations -- a real governance relationship Maleficent never has here). Narrative Acceptance of Injustice (0) since the ending fully undoes all harm. Explicit Darkness (2) for real, sustained peril (the curse, Maleficent's dragon-form battle, the thorn forest) without graphic content, consistent with this catalog's other Tier 1-2 Disney entries. Compared against Maleficent (2014, Tier 3, 3.3, SD0/LH0/MC1/SC1/RD1/NAI1/ED2), the live-action reinterpretation deliberately adds real moral cynicism, structural corruption (Stefan's own rule turns paranoid/tyrannical), redemption difficulty, and narrative injustice (the wing-severing assault) that the 1959 original doesn't carry -- the same 'source vs. dark reimagining' relationship already established elsewhere in this catalog (The Wizard of Oz vs. Wicked, Journey to the West vs. Black Myth: Wukong). The darkest entry currently in Tier 1, just 0.05 below the Tier 2 threshold.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cinderella</t>
+  </si>
+  <si>
+    <t xml:space="preserve">genre gate trivial -- the Fairy Godmother's transformation magic (pumpkin to coach, mice to horses, rags to gown) and its midnight time-limit curse are the entire second act's driving mechanism, not decoration. Structural Despair (0) since the years of servitude are fully and permanently undone by the ending. Limited Heroism (0) since the victory is complete -- nothing is left compromised for Cinderella. Moral Cynicism (1) since the stepfamily materially benefits from years of unpaid forced labor extracted from Cinderella, a real sustained reward for cruelty only reversed at the very end -- parallels Frozen's Hans (wrongdoing rewarded, then fully stopped). Structural Corruption (0): this is household-scale, single-victim cruelty backed by ordinary guardian authority, not governance over a subject population or a genuine institution (contrast The Wizard of Oz and Alice in Wonderland (2010-2016), both SC=2, or Encanto's village-founding dynasty, SC=1) -- matches the 'personal betrayal, no institution examined' read used for Puss in Boots (2011). Redemption Difficulty (0) since no character atones for real wrongdoing. Narrative Acceptance of Injustice (0) since Cinderella's own core injustice is fully and durably resolved, and the stepfamily isn't left as an ongoing threat (unlike Rise of the Guardians' Pitch). Explicit Darkness (2) for real but contained cruelty/peril (imprisonment, drudgery, fear) without graphic content, consistent with this catalog's other Tier 1-2 Disney entries. Exact 7-axis profile match with Frozen (2013); score tie with Hercules and Moana via different profiles.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2274,7 +2280,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R157"/>
+  <dimension ref="A1:R158"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -10776,7 +10782,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="1" t="n">
         <v>1</v>
       </c>
@@ -10830,6 +10836,62 @@
       </c>
       <c r="R157" s="1" t="s">
         <v>479</v>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B158" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C158" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="D158" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E158" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F158" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G158" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H158" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I158" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J158" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K158" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L158" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M158" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N158" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O158" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P158" s="1" t="n">
+        <v>2.2875</v>
+      </c>
+      <c r="Q158" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R158" s="1" t="s">
+        <v>481</v>
       </c>
     </row>
   </sheetData>
@@ -10864,7 +10926,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10886,7 +10948,7 @@
         <v>82</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10979,7 +11041,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Aladdin (1992) to Tier 2
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1144" uniqueCount="486">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1468,6 +1468,12 @@
   </si>
   <si>
     <t xml:space="preserve">genre gate trivial -- the Fairy Godmother's transformation magic (pumpkin to coach, mice to horses, rags to gown) and its midnight time-limit curse are the entire second act's driving mechanism, not decoration. Structural Despair (0) since the years of servitude are fully and permanently undone by the ending. Limited Heroism (0) since the victory is complete -- nothing is left compromised for Cinderella. Moral Cynicism (1) since the stepfamily materially benefits from years of unpaid forced labor extracted from Cinderella, a real sustained reward for cruelty only reversed at the very end -- parallels Frozen's Hans (wrongdoing rewarded, then fully stopped). Structural Corruption (0): this is household-scale, single-victim cruelty backed by ordinary guardian authority, not governance over a subject population or a genuine institution (contrast The Wizard of Oz and Alice in Wonderland (2010-2016), both SC=2, or Encanto's village-founding dynasty, SC=1) -- matches the 'personal betrayal, no institution examined' read used for Puss in Boots (2011). Redemption Difficulty (0) since no character atones for real wrongdoing. Narrative Acceptance of Injustice (0) since Cinderella's own core injustice is fully and durably resolved, and the stepfamily isn't left as an ongoing threat (unlike Rise of the Guardians' Pitch). Explicit Darkness (2) for real but contained cruelty/peril (imprisonment, drudgery, fear) without graphic content, consistent with this catalog's other Tier 1-2 Disney entries. Exact 7-axis profile match with Frozen (2013); score tie with Hercules and Moana via different profiles.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aladdin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">genre gate trivial -- a genie with real wish-granting magic, a sorcerer villain (Jafar) who performs real magic and transforms into a giant cobra then a genie himself, a living magic carpet, a wish-granting lamp, the Cave of Wonders -- magic is the entire plot engine. Structural Despair (0) since Aladdin's poverty is fully and permanently resolved by the ending. Limited Heroism (0) since Jafar is completely defeated and the Sultan's law changes fully, not partially. Moral Cynicism (1) since Jafar, the Sultan's own trusted royal vizier, hypnotizes and controls the legitimate ruler for a real stretch of the film and briefly seizes absolute power -- a genuine, if temporary, reward for treachery from a position of real trust. Structural Corruption (1) since Jafar doesn't just scheme -- he actively usurps the throne, commandeers the palace guard, and declares himself absolute ruler, a real institutional capture, but brief and same-day reversed (contrast the sustained tyrannies that earned The Wizard of Oz and Alice in Wonderland (2010-2016) SC=2). Redemption Difficulty (0) since no character atones for real wrongdoing -- Aladdin's 'Prince Ali' lie is minor and costs him nothing when revealed. Narrative Acceptance of Injustice (1) since Jafar isn't destroyed, only trapped in his lamp and banished -- a real loose end the story itself leaves open (and the sequel confirms he returns), paralleling Rise of the Guardians' Pitch. Explicit Darkness (2) for intense magical peril (the cobra transformation, the sorcerer battle, an engulfing sandstorm) but no on-screen death or graphic violence -- re-benchmarked against Alice in Wonderland (2010-2016), which scored ED=2 despite on-screen executions and a graphic decapitation, this doesn't clear that bar. Exact 7-axis profile tie with the existing 2.9625 cluster (Puss in Boots (2011), DanMachi, The Chronicles of Narnia, The Legend of Zelda, The Princess Bride, Journey to the West), each via a different distribution.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2280,7 +2286,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R158"/>
+  <dimension ref="A1:R159"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -10838,7 +10844,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="1" t="n">
         <v>2</v>
       </c>
@@ -10892,6 +10898,62 @@
       </c>
       <c r="R158" s="1" t="s">
         <v>481</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B159" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="D159" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E159" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F159" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G159" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H159" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I159" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J159" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K159" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L159" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M159" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N159" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O159" s="1" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="P159" s="1" t="n">
+        <v>2.9625</v>
+      </c>
+      <c r="Q159" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R159" s="1" t="s">
+        <v>483</v>
       </c>
     </row>
   </sheetData>
@@ -10926,7 +10988,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10948,7 +11010,7 @@
         <v>82</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11041,7 +11103,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Sorcerer's Apprentice (2010) to Tier 2
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1144" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1151" uniqueCount="488">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1474,6 +1474,12 @@
   </si>
   <si>
     <t xml:space="preserve">genre gate trivial -- a genie with real wish-granting magic, a sorcerer villain (Jafar) who performs real magic and transforms into a giant cobra then a genie himself, a living magic carpet, a wish-granting lamp, the Cave of Wonders -- magic is the entire plot engine. Structural Despair (0) since Aladdin's poverty is fully and permanently resolved by the ending. Limited Heroism (0) since Jafar is completely defeated and the Sultan's law changes fully, not partially. Moral Cynicism (1) since Jafar, the Sultan's own trusted royal vizier, hypnotizes and controls the legitimate ruler for a real stretch of the film and briefly seizes absolute power -- a genuine, if temporary, reward for treachery from a position of real trust. Structural Corruption (1) since Jafar doesn't just scheme -- he actively usurps the throne, commandeers the palace guard, and declares himself absolute ruler, a real institutional capture, but brief and same-day reversed (contrast the sustained tyrannies that earned The Wizard of Oz and Alice in Wonderland (2010-2016) SC=2). Redemption Difficulty (0) since no character atones for real wrongdoing -- Aladdin's 'Prince Ali' lie is minor and costs him nothing when revealed. Narrative Acceptance of Injustice (1) since Jafar isn't destroyed, only trapped in his lamp and banished -- a real loose end the story itself leaves open (and the sequel confirms he returns), paralleling Rise of the Guardians' Pitch. Explicit Darkness (2) for intense magical peril (the cobra transformation, the sorcerer battle, an engulfing sandstorm) but no on-screen death or graphic violence -- re-benchmarked against Alice in Wonderland (2010-2016), which scored ED=2 despite on-screen executions and a graphic decapitation, this doesn't clear that bar. Exact 7-axis profile tie with the existing 2.9625 cluster (Puss in Boots (2011), DanMachi, The Chronicles of Narnia, The Legend of Zelda, The Princess Bride, Journey to the West), each via a different distribution.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Sorcerer's Apprentice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">genre gate trivial -- Merlin, Morgana le Fay, and real wizard-apprentice combat magic are the entire premise (the Grimhold, plasma-bolt duels, the 'Rising' resurrection spell). Structural Despair (0) since the magical conflict is a contained secret-order struggle inside an otherwise ordinary present-day world, not a world-level decay. Limited Heroism (0) since the apocalyptic Rising is fully and permanently prevented -- Morgana is destroyed outright by Dave's plasma attack, not merely contained. Moral Cynicism (1) since Horvath's deception of a child (young Dave, tricked into freeing him from the Grimhold in 2000) lets him trap Balthazar in an urn for a full decade before the main story even begins -- a real, sustained win for treachery, not a same-day-reversed scheme. Structural Corruption (0) since no institution is examined -- the Merlinean/Morganian conflict is a small secret order, not a governing body. Redemption Difficulty (0) since no character arc centers on atoning for real wrongdoing; Dave's arc is coming-of-age, not redemption. Narrative Acceptance of Injustice (1) since Horvath survives and escapes at the very end (confirmed in the post-credits stinger) -- a real loose end the story itself leaves open, the same shape as Aladdin's Jafar and Rise of the Guardians' Pitch. Explicit Darkness (2) for real magical peril (a living dragon statue's rampage through Chinatown, Tesla-coil plasma battles, Balthazar's temporary death) without graphic detail, consistent with this catalog's other Tier 1-2 Disney entries. Weighted = 0.5, Final Score = 2.625, exact score tie with Harry Potter and the Chamber of Secrets, The Wizard of Oz, The Little Prince, and Onward, each via a different profile -- closest match is Chamber of Secrets (Structural Corruption 1 + Narrative Acceptance of Injustice 1 there vs. Moral Cynicism 1 + Narrative Acceptance of Injustice 1 here). Cozy Fantasy = No, Hopepunk = No (no societal oppression + resistance shape, just a personal villain threat). Label check: 'Bright Fantasy' fits -- a decisively triumphant mentor/apprentice adventure with one contained villain loose end.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2286,7 +2292,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R159"/>
+  <dimension ref="A1:R160"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -10900,7 +10906,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="1" t="n">
         <v>2</v>
       </c>
@@ -10954,6 +10960,62 @@
       </c>
       <c r="R159" s="1" t="s">
         <v>483</v>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B160" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="D160" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E160" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F160" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G160" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H160" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I160" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K160" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L160" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M160" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N160" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O160" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P160" s="1" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="Q160" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R160" s="1" t="s">
+        <v>485</v>
       </c>
     </row>
   </sheetData>
@@ -10988,7 +11050,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11103,7 +11165,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Raya and the Last Dragon (2021) to Tier 2
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1151" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1158" uniqueCount="490">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1480,6 +1480,12 @@
   </si>
   <si>
     <t xml:space="preserve">genre gate trivial -- Merlin, Morgana le Fay, and real wizard-apprentice combat magic are the entire premise (the Grimhold, plasma-bolt duels, the 'Rising' resurrection spell). Structural Despair (0) since the magical conflict is a contained secret-order struggle inside an otherwise ordinary present-day world, not a world-level decay. Limited Heroism (0) since the apocalyptic Rising is fully and permanently prevented -- Morgana is destroyed outright by Dave's plasma attack, not merely contained. Moral Cynicism (1) since Horvath's deception of a child (young Dave, tricked into freeing him from the Grimhold in 2000) lets him trap Balthazar in an urn for a full decade before the main story even begins -- a real, sustained win for treachery, not a same-day-reversed scheme. Structural Corruption (0) since no institution is examined -- the Merlinean/Morganian conflict is a small secret order, not a governing body. Redemption Difficulty (0) since no character arc centers on atoning for real wrongdoing; Dave's arc is coming-of-age, not redemption. Narrative Acceptance of Injustice (1) since Horvath survives and escapes at the very end (confirmed in the post-credits stinger) -- a real loose end the story itself leaves open, the same shape as Aladdin's Jafar and Rise of the Guardians' Pitch. Explicit Darkness (2) for real magical peril (a living dragon statue's rampage through Chinatown, Tesla-coil plasma battles, Balthazar's temporary death) without graphic detail, consistent with this catalog's other Tier 1-2 Disney entries. Weighted = 0.5, Final Score = 2.625, exact score tie with Harry Potter and the Chamber of Secrets, The Wizard of Oz, The Little Prince, and Onward, each via a different profile -- closest match is Chamber of Secrets (Structural Corruption 1 + Narrative Acceptance of Injustice 1 there vs. Moral Cynicism 1 + Narrative Acceptance of Injustice 1 here). Cozy Fantasy = No, Hopepunk = No (no societal oppression + resistance shape, just a personal villain threat). Label check: 'Bright Fantasy' fits -- a decisively triumphant mentor/apprentice adventure with one contained villain loose end.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raya and the Last Dragon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENRE GATE: dragons, a magic gem, and the Druun mythology (mindless spirits that petrify all living things) drive the entire plot; not a fantasy-adjacent adventure but core fantasy, clears the strict gate easily. SD=0: Kumandra is a 500-year-old static political fracture, not an actively decaying trajectory independent of the plot; the world is not shown trending toward decline on its own. LH=0: the ending is a full structural reset -- the Druun are permanently vanquished, all petrified victims and the dragons are revived, and the five nations reunify as one land; heroism changes the background structure unambiguously. MC=1: Fang's isolationist hoarding of its gem shard visibly buys it real, lasting material advantage (clean water, comfort) while other nations suffer for years -- self-interest pays off practically even though the film ultimately condemns it. SC=0: no central institution is designed to perpetuate injustice; the conflict is inter-tribal distrust and war, not institutional corruption. RD=2: both Namaari's and Raya's redemption arcs cost something real -- Raya's own lingering distrust directly causes Sisu's death, and reconciliation only comes after that genuine loss. NAI=0: every harm (deaths, petrification, political division) is fully and explicitly undone by the ending -- injustice is treated as entirely temporary. ED=2: real physical combat and visible peril (petrification, dissolution to dust) without extreme graphic detail. Neighbor check: lands at 2.9625, matching Aladdin exactly via a different profile (MC1/RD2/NAI0 vs. MC1/SC1/NAI1) -- both villain-driven Disney adventures with total resolution. Comfortably below the lowest Tier 3 works (Mushishi, A Choir of Lies, Neverwinter Nights, Puss in Boots: The Last Wish), which all stack an SD/LH/RD&gt;=1 axis with heavier Explicit Darkness.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2292,7 +2298,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R160"/>
+  <dimension ref="A1:R161"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -10962,7 +10968,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="1" t="n">
         <v>2</v>
       </c>
@@ -11016,6 +11022,62 @@
       </c>
       <c r="R160" s="1" t="s">
         <v>485</v>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C161" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="D161" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E161" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F161" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G161" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H161" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I161" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K161" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L161" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M161" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N161" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O161" s="1" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="P161" s="1" t="n">
+        <v>2.9625</v>
+      </c>
+      <c r="Q161" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R161" s="1" t="s">
+        <v>487</v>
       </c>
     </row>
   </sheetData>
@@ -11050,7 +11112,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11165,7 +11227,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Pirates of the Caribbean (2003-2007) to Tier 4
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1158" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1165" uniqueCount="492">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1486,6 +1486,12 @@
   </si>
   <si>
     <t xml:space="preserve">GENRE GATE: dragons, a magic gem, and the Druun mythology (mindless spirits that petrify all living things) drive the entire plot; not a fantasy-adjacent adventure but core fantasy, clears the strict gate easily. SD=0: Kumandra is a 500-year-old static political fracture, not an actively decaying trajectory independent of the plot; the world is not shown trending toward decline on its own. LH=0: the ending is a full structural reset -- the Druun are permanently vanquished, all petrified victims and the dragons are revived, and the five nations reunify as one land; heroism changes the background structure unambiguously. MC=1: Fang's isolationist hoarding of its gem shard visibly buys it real, lasting material advantage (clean water, comfort) while other nations suffer for years -- self-interest pays off practically even though the film ultimately condemns it. SC=0: no central institution is designed to perpetuate injustice; the conflict is inter-tribal distrust and war, not institutional corruption. RD=2: both Namaari's and Raya's redemption arcs cost something real -- Raya's own lingering distrust directly causes Sisu's death, and reconciliation only comes after that genuine loss. NAI=0: every harm (deaths, petrification, political division) is fully and explicitly undone by the ending -- injustice is treated as entirely temporary. ED=2: real physical combat and visible peril (petrification, dissolution to dust) without extreme graphic detail. Neighbor check: lands at 2.9625, matching Aladdin exactly via a different profile (MC1/RD2/NAI0 vs. MC1/SC1/NAI1) -- both villain-driven Disney adventures with total resolution. Comfortably below the lowest Tier 3 works (Mushishi, A Choir of Lies, Neverwinter Nights, Puss in Boots: The Last Wish), which all stack an SD/LH/RD&gt;=1 axis with heavier Explicit Darkness.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pirates of the Caribbean (2003-2007)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCOPE: original trilogy only (Curse of the Black Pearl 2003, Dead Man's Chest 2006, At World's End 2007) scored as one entry, following the Lord of the Rings precedent (one continuous story, consistent tone); On Stranger Tides (2011) and Dead Men Tell No Tales (2017) excluded. GENRE GATE: real Aztec curse (moonlit skeleton crew), Davy Jones and the cursed Flying Dutchman crew, the Kraken, sea goddess Calypso bound in human form; load-bearing supernatural content, clears the strict gate. SD=1: piracy's free era being squeezed by corporate/colonial consolidation is a real but subtextual throughline, not a dominant baked-in decline. LH=1: Beckett dies and his fleet is destroyed (real, fairly lasting victory); the broader march of empire is left as a minor open note in the elegiac coda. MC=1: ruthless self-interest (Beckett, Barbossa) buys real temporary power, but the story is ultimately a just-world narrative; virtue vindicated, cruelty punished. SC=2: the East India Trading Company is corrupt by design, but the Pirate Brethren Court stands as a functioning legitimate alternative. RD=2: Norrington's redemption (betrays principles for ambition, then redeems himself through a fatal sacrifice) costs his life. NAI=1: the specific injustice (Beckett's tyranny) is decisively resolved; the broader wistfulness about piracy's fading era is tonal color. ED=3: frequent visible horror content across all three films (skeleton crews, Kraken, tentacled Davy Jones/Dutchman crew) without extreme graphic detail. Neighbor check: exact profile match with Fullmetal Alchemist: Brotherhood (4.875); also alongside Final Fantasy IX, Ranking of Kings, Shannara Chronicles, Vox Machina. Lowest Tier 5 works all carry SD2 or ED4.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2298,7 +2304,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R161"/>
+  <dimension ref="A1:R162"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -11024,7 +11030,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="1" t="n">
         <v>2</v>
       </c>
@@ -11078,6 +11084,62 @@
       </c>
       <c r="R161" s="1" t="s">
         <v>487</v>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B162" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C162" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="D162" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="E162" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F162" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G162" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H162" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I162" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J162" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K162" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L162" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M162" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N162" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O162" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P162" s="1" t="n">
+        <v>4.875</v>
+      </c>
+      <c r="Q162" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="R162" s="1" t="s">
+        <v>489</v>
       </c>
     </row>
   </sheetData>
@@ -11112,7 +11174,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11227,7 +11289,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Mary Poppins (1964) to Tier 1
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1165" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1172" uniqueCount="494">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1492,6 +1492,12 @@
   </si>
   <si>
     <t xml:space="preserve">SCOPE: original trilogy only (Curse of the Black Pearl 2003, Dead Man's Chest 2006, At World's End 2007) scored as one entry, following the Lord of the Rings precedent (one continuous story, consistent tone); On Stranger Tides (2011) and Dead Men Tell No Tales (2017) excluded. GENRE GATE: real Aztec curse (moonlit skeleton crew), Davy Jones and the cursed Flying Dutchman crew, the Kraken, sea goddess Calypso bound in human form; load-bearing supernatural content, clears the strict gate. SD=1: piracy's free era being squeezed by corporate/colonial consolidation is a real but subtextual throughline, not a dominant baked-in decline. LH=1: Beckett dies and his fleet is destroyed (real, fairly lasting victory); the broader march of empire is left as a minor open note in the elegiac coda. MC=1: ruthless self-interest (Beckett, Barbossa) buys real temporary power, but the story is ultimately a just-world narrative; virtue vindicated, cruelty punished. SC=2: the East India Trading Company is corrupt by design, but the Pirate Brethren Court stands as a functioning legitimate alternative. RD=2: Norrington's redemption (betrays principles for ambition, then redeems himself through a fatal sacrifice) costs his life. NAI=1: the specific injustice (Beckett's tyranny) is decisively resolved; the broader wistfulness about piracy's fading era is tonal color. ED=3: frequent visible horror content across all three films (skeleton crews, Kraken, tentacled Davy Jones/Dutchman crew) without extreme graphic detail. Neighbor check: exact profile match with Fullmetal Alchemist: Brotherhood (4.875); also alongside Final Fantasy IX, Ranking of Kings, Shannara Chronicles, Vox Machina. Lowest Tier 5 works all carry SD2 or ED4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mary Poppins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENRE GATE: flight via umbrella, a bottomless carpet bag, entering an animated chalk-drawing world, a tea party on the ceiling -- magic drives multiple full sequences, not incidental whimsy; clears the strict gate. RELEVANCE: passes -- the story is built around a magical nanny's interventions, not a mundane drama with decorative fantasy trim. All axes 0: SD=0 (idealized, cheerful Edwardian London, no decay theme). LH=0 (the family's dysfunction is fully and permanently resolved -- complete reconciliation, no loose ends). MC=0 (no scheming/villainy to test; kindness and honesty are directly, immediately rewarded -- Dawes Sr. literally floats with joy at George's good humor). SC=0 (the bank isn't corrupt, just impersonal -- a misplaced-values problem corrected amicably, not an institutional injustice). RD=0 (George's workaholic neglect is fixed with essentially no dramatic cost). NAI=0 (no real injustice is ever present to accept or resolve). ED=0 (zero physical danger -- the bank-run scene is social/emotional chaos, not violence or threat; per critical consensus the film has "no real peril"). Neighbor check: exact all-zero tie with My Neighbor Totoro, Kiki's Delivery Service, Ponyo, and Legends &amp; Lattes -- the catalog's wholesome floor. Sits below Sleeping Beauty (1.95, ED2, an actual curse/dragon-battle threat), correctly, since Mary Poppins has even less peril.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2304,7 +2310,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R162"/>
+  <dimension ref="A1:R163"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -11086,7 +11092,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="1" t="n">
         <v>4</v>
       </c>
@@ -11140,6 +11146,62 @@
       </c>
       <c r="R162" s="1" t="s">
         <v>489</v>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B163" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="D163" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E163" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F163" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G163" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H163" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I163" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J163" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K163" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L163" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M163" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N163" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O163" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P163" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Q163" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R163" s="1" t="s">
+        <v>491</v>
       </c>
     </row>
   </sheetData>
@@ -11174,7 +11236,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11289,7 +11351,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Enchanted (2007) to Tier 2
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1172" uniqueCount="494">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1179" uniqueCount="496">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1498,6 +1498,12 @@
   </si>
   <si>
     <t xml:space="preserve">GENRE GATE: flight via umbrella, a bottomless carpet bag, entering an animated chalk-drawing world, a tea party on the ceiling -- magic drives multiple full sequences, not incidental whimsy; clears the strict gate. RELEVANCE: passes -- the story is built around a magical nanny's interventions, not a mundane drama with decorative fantasy trim. All axes 0: SD=0 (idealized, cheerful Edwardian London, no decay theme). LH=0 (the family's dysfunction is fully and permanently resolved -- complete reconciliation, no loose ends). MC=0 (no scheming/villainy to test; kindness and honesty are directly, immediately rewarded -- Dawes Sr. literally floats with joy at George's good humor). SC=0 (the bank isn't corrupt, just impersonal -- a misplaced-values problem corrected amicably, not an institutional injustice). RD=0 (George's workaholic neglect is fixed with essentially no dramatic cost). NAI=0 (no real injustice is ever present to accept or resolve). ED=0 (zero physical danger -- the bank-run scene is social/emotional chaos, not violence or threat; per critical consensus the film has "no real peril"). Neighbor check: exact all-zero tie with My Neighbor Totoro, Kiki's Delivery Service, Ponyo, and Legends &amp; Lattes -- the catalog's wholesome floor. Sits below Sleeping Beauty (1.95, ED2, an actual curse/dragon-battle threat), correctly, since Mary Poppins has even less peril.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enchanted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENRE GATE: a real sorceress-queen (Narissa) with genuine curse, transformation, and portal magic -- a magic portal between the 2D animated fantasy kingdom of Andalasia and live-action New York, a poisoned-apple sleeping curse, and a climactic dragon transformation; load-bearing fantasy, clears the strict gate easily, same "wicked queen with real magic and a dragon-transformation climax" shape as Sleeping Beauty. SD=0: Giselle's exile resolves into a thriving new life; nothing is left in decline. LH=0: complete, unambiguous victory -- Narissa defeated, Giselle/Robert together, Edward/Nancy married, nothing compromised. MC=1: Narissa retains her throne throughout the film precisely because of her scheming (banishment, then the poisoned-apple murder attempt), a real if temporary reward for wrongdoing, undone only at the very end -- parallels Cinderella's stepfamily read. SC=0: a personal/dynastic succession conflict, not depicted institutional oppression of Andalasia's subjects -- matches Sleeping Beauty/Cinderella precedent, contrast Wizard of Oz's SC2 enslaved Winkies. RD=1: Nathaniel commits genuine wrongdoing (attempted poisoning on Narissa's orders) and atones by exposing her plot, resolved without extreme cost -- parallels Spirited Away's No-Face. NAI=0: nothing left unresolved; full happy-ending reset. ED=2: real peril (the poisoning, the dragon battle, a villain's death) without graphic content, consistent with this catalog's Tier 1-2 Disney band (Sleeping Beauty, Aladdin, Wizard of Oz). Neighbor check: lands at 2.625, an exact score tie with Onward, Wizard of Oz, Alice in Wonderland (2010-2016), and Harry Potter and the Chamber of Secrets, all via different profiles. Label check: "Bright Fantasy" fits.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2310,7 +2316,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R163"/>
+  <dimension ref="A1:R164"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -11148,7 +11154,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="1" t="n">
         <v>1</v>
       </c>
@@ -11202,6 +11208,62 @@
       </c>
       <c r="R163" s="1" t="s">
         <v>491</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B164" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="D164" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E164" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F164" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G164" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H164" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I164" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J164" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K164" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L164" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M164" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N164" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O164" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P164" s="1" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="Q164" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R164" s="1" t="s">
+        <v>493</v>
       </c>
     </row>
   </sheetData>
@@ -11236,7 +11298,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11351,7 +11413,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Tangled (2010) to Tier 3
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1179" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="498">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1504,6 +1504,12 @@
   </si>
   <si>
     <t xml:space="preserve">GENRE GATE: a real sorceress-queen (Narissa) with genuine curse, transformation, and portal magic -- a magic portal between the 2D animated fantasy kingdom of Andalasia and live-action New York, a poisoned-apple sleeping curse, and a climactic dragon transformation; load-bearing fantasy, clears the strict gate easily, same "wicked queen with real magic and a dragon-transformation climax" shape as Sleeping Beauty. SD=0: Giselle's exile resolves into a thriving new life; nothing is left in decline. LH=0: complete, unambiguous victory -- Narissa defeated, Giselle/Robert together, Edward/Nancy married, nothing compromised. MC=1: Narissa retains her throne throughout the film precisely because of her scheming (banishment, then the poisoned-apple murder attempt), a real if temporary reward for wrongdoing, undone only at the very end -- parallels Cinderella's stepfamily read. SC=0: a personal/dynastic succession conflict, not depicted institutional oppression of Andalasia's subjects -- matches Sleeping Beauty/Cinderella precedent, contrast Wizard of Oz's SC2 enslaved Winkies. RD=1: Nathaniel commits genuine wrongdoing (attempted poisoning on Narissa's orders) and atones by exposing her plot, resolved without extreme cost -- parallels Spirited Away's No-Face. NAI=0: nothing left unresolved; full happy-ending reset. ED=2: real peril (the poisoning, the dragon battle, a villain's death) without graphic content, consistent with this catalog's Tier 1-2 Disney band (Sleeping Beauty, Aladdin, Wizard of Oz). Neighbor check: lands at 2.625, an exact score tie with Onward, Wizard of Oz, Alice in Wonderland (2010-2016), and Harry Potter and the Chamber of Secrets, all via different profiles. Label check: "Bright Fantasy" fits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tangled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENRE GATE: Rapunzel's hair has real, functioning magic (genuine healing/youth-restoring power when sung to, lost permanently if cut) that is the entire reason Mother Gothel keeps her captive and the mechanism of the climax; load-bearing, clears the strict gate easily. SD=0: personal-scale abduction/imprisonment, not a broader societal decline; fully resolved. LH=0: complete, unambiguous victory -- Rapunzel freed and reunited with her family, Flynn survives and is pardoned, Gothel destroyed. MC=1: Gothel benefits materially (eternal youth) from 18 years of abduction and psychological abuse, a real sustained reward for wrongdoing, undone only at her death -- parallels Cinderella's stepfamily read. SC=0: single-victim, personal-scale cruelty, not institutional oppression of a population (matches Cinderella/Sleeping Beauty precedent). RD=2: Flynn's redemption is genuinely costly -- he deliberately destroys Rapunzel's only means to heal his fatal wound in order to free her, choosing her freedom over his own life; parallels Norrington's fatal sacrifice in Pirates of the Caribbean. NAI=0: full resolution; nothing left unaddressed. ED=3: an on-screen stabbing, a villain's visible death (rapid aging, crumbling to dust), and 18 years of sustained psychological imprisonment; comparable to Rise of the Guardians' ED3, above the ED2 contained-peril ceiling of Sleeping Beauty/Aladdin/Enchanted. Neighbor check: 3.1875 shares its exact score with Return to Oz via a very different profile; sits between Neverwinter Nights/A Choir of Lies/Mushishi (3.075) and Dungeon Meshi/Cormyr/Maleficent (3.30). Boundary check: WIS 0.75 clears the Tier 3 floor (0.667) comfortably. Label check: "Moderately Bright Fantasy" fits.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2316,7 +2322,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R164"/>
+  <dimension ref="A1:R165"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -11210,7 +11216,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="1" t="n">
         <v>2</v>
       </c>
@@ -11264,6 +11270,62 @@
       </c>
       <c r="R164" s="1" t="s">
         <v>493</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B165" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C165" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="D165" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E165" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F165" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G165" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H165" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I165" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J165" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K165" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L165" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="M165" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N165" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O165" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P165" s="1" t="n">
+        <v>3.1875</v>
+      </c>
+      <c r="Q165" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="R165" s="1" t="s">
+        <v>495</v>
       </c>
     </row>
   </sheetData>
@@ -11298,7 +11360,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11413,7 +11475,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Brave (2012) to Tier 2
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="500">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1510,6 +1510,12 @@
   </si>
   <si>
     <t xml:space="preserve">GENRE GATE: Rapunzel's hair has real, functioning magic (genuine healing/youth-restoring power when sung to, lost permanently if cut) that is the entire reason Mother Gothel keeps her captive and the mechanism of the climax; load-bearing, clears the strict gate easily. SD=0: personal-scale abduction/imprisonment, not a broader societal decline; fully resolved. LH=0: complete, unambiguous victory -- Rapunzel freed and reunited with her family, Flynn survives and is pardoned, Gothel destroyed. MC=1: Gothel benefits materially (eternal youth) from 18 years of abduction and psychological abuse, a real sustained reward for wrongdoing, undone only at her death -- parallels Cinderella's stepfamily read. SC=0: single-victim, personal-scale cruelty, not institutional oppression of a population (matches Cinderella/Sleeping Beauty precedent). RD=2: Flynn's redemption is genuinely costly -- he deliberately destroys Rapunzel's only means to heal his fatal wound in order to free her, choosing her freedom over his own life; parallels Norrington's fatal sacrifice in Pirates of the Caribbean. NAI=0: full resolution; nothing left unaddressed. ED=3: an on-screen stabbing, a villain's visible death (rapid aging, crumbling to dust), and 18 years of sustained psychological imprisonment; comparable to Rise of the Guardians' ED3, above the ED2 contained-peril ceiling of Sleeping Beauty/Aladdin/Enchanted. Neighbor check: 3.1875 shares its exact score with Return to Oz via a very different profile; sits between Neverwinter Nights/A Choir of Lies/Mushishi (3.075) and Dungeon Meshi/Cormyr/Maleficent (3.30). Boundary check: WIS 0.75 clears the Tier 3 floor (0.667) comfortably. Label check: "Moderately Bright Fantasy" fits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brave</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENRE GATE: a witch's enchanted cake transforms Queen Elinor into a bear and drives the whole plot; will-o'-the-wisps are real magical guides and the cursed-prince legend (Mor'du) is confirmed true within the story; load-bearing, clears the strict gate. RELEVANCE: passes. SD=0: a family conflict, not a declining world; fully resolved. LH=0: curse broken, Mor'du destroyed, betrothal custom reformed -- complete victory. MC=0: nobody profits from wrongdoing; Merida's selfish act has real consequences and Mor'du's pride cost him everything. SC=0: the betrothal custom is a rigid tradition, not an institution built to perpetuate harm, and it is reformed by the end (Cinderella/Sleeping Beauty read); 1 considered and rejected. RD=1: Merida must face real guilt and repair what she broke under a deadline with a genuine risk of permanent loss, but nothing is actually lost and there is no fatal sacrifice (contrast Flynn/Norrington RD2). NAI=0: everything is undone or resolved by the ending. ED=2: real peril (Mor'du's attacks, Elinor losing her humanity, Mor'du's death) without graphic content; 3 ruled out -- no on-screen stabbing or sustained abuse as in Tangled. Neighbor check: 2.2875 ties Cinderella, Frozen, Hercules, Moana, Castle in the Sky, Labyrinth, The Addams Family (1964-1992) via different profiles (RD1 instead of Cinderella's MC1). Boundary check: WIS 0.35 well above the Tier 2 floor (0.222). Label check: "Bright Fantasy" fits.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2322,7 +2328,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R165"/>
+  <dimension ref="A1:R166"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -11272,7 +11278,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="1" t="n">
         <v>3</v>
       </c>
@@ -11326,6 +11332,62 @@
       </c>
       <c r="R165" s="1" t="s">
         <v>495</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C166" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="D166" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E166" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="F166" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G166" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H166" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I166" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J166" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K166" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L166" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M166" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N166" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O166" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P166" s="1" t="n">
+        <v>2.2875</v>
+      </c>
+      <c r="Q166" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R166" s="1" t="s">
+        <v>497</v>
       </c>
     </row>
   </sheetData>
@@ -11360,7 +11422,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11475,7 +11537,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Sword in the Stone (1963) to Tier 1; queue The Black Cauldron
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="502">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1516,6 +1516,12 @@
   </si>
   <si>
     <t xml:space="preserve">GENRE GATE: a witch's enchanted cake transforms Queen Elinor into a bear and drives the whole plot; will-o'-the-wisps are real magical guides and the cursed-prince legend (Mor'du) is confirmed true within the story; load-bearing, clears the strict gate. RELEVANCE: passes. SD=0: a family conflict, not a declining world; fully resolved. LH=0: curse broken, Mor'du destroyed, betrothal custom reformed -- complete victory. MC=0: nobody profits from wrongdoing; Merida's selfish act has real consequences and Mor'du's pride cost him everything. SC=0: the betrothal custom is a rigid tradition, not an institution built to perpetuate harm, and it is reformed by the end (Cinderella/Sleeping Beauty read); 1 considered and rejected. RD=1: Merida must face real guilt and repair what she broke under a deadline with a genuine risk of permanent loss, but nothing is actually lost and there is no fatal sacrifice (contrast Flynn/Norrington RD2). NAI=0: everything is undone or resolved by the ending. ED=2: real peril (Mor'du's attacks, Elinor losing her humanity, Mor'du's death) without graphic content; 3 ruled out -- no on-screen stabbing or sustained abuse as in Tangled. Neighbor check: 2.2875 ties Cinderella, Frozen, Hercules, Moana, Castle in the Sky, Labyrinth, The Addams Family (1964-1992) via different profiles (RD1 instead of Cinderella's MC1). Boundary check: WIS 0.35 well above the Tier 2 floor (0.222). Label check: "Bright Fantasy" fits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Sword in the Stone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENRE GATE: Merlin is a practicing wizard whose transformation magic (Wart as fish, squirrel, sparrow) and the wizards' duel with Madam Mim are among the most extensive in the classic Disney line; the sword in the stone is a real magical test of destiny; load-bearing, clears the strict gate easily. RELEVANCE: passes. SD=0: no societal decline; Uther's missing heir is a plot setup that Arthur's coronation fully resolves. LH=0: the sword is pulled, the prophecy is fulfilled, and Merlin returns to help; Arthur's self-doubt is a mild beat, not an unresolved loss. MC=0: nobody profits from wrongdoing and Mim is defeated; Ector's servant-like treatment of Wart is minor and ends in an apology. SC=0: no institution examined. RD=0: no one atones for real wrongdoing. NAI=0: nothing left unresolved. ED=1: G-rated, no deaths or graphic content; peril (pike, wolf, hawk, Mim's capture of Wart) is played comically, and Mim's dragon form comes in a gag-driven duel; below Sleeping Beauty's ED2 where the curse and dragon battle are treated seriously. Neighbor check: 1.725 is an exact 7-axis profile match with Final Fantasy I (ED1 only); Mary Poppins/Totoro/Kiki (1.5, all zeros) sit below and Sleeping Beauty (1.95, ED2) above. Boundary check: WIS 0.10 is far from the Tier 2 floor (0.222). Label check: "Very Bright Fantasy" fits.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2328,7 +2334,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R166"/>
+  <dimension ref="A1:R167"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -11334,7 +11340,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="1" t="n">
         <v>2</v>
       </c>
@@ -11388,6 +11394,62 @@
       </c>
       <c r="R166" s="1" t="s">
         <v>497</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B167" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C167" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="D167" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E167" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F167" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G167" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H167" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I167" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J167" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K167" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L167" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M167" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N167" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O167" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="P167" s="1" t="n">
+        <v>1.725</v>
+      </c>
+      <c r="Q167" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R167" s="1" t="s">
+        <v>499</v>
       </c>
     </row>
   </sheetData>
@@ -11422,7 +11484,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11537,7 +11599,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Miss Peregrine's Home for Peculiar Children (2011 novel) to Tier 3; queue the 2016 film
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="505">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1522,6 +1522,15 @@
   </si>
   <si>
     <t xml:space="preserve">GENRE GATE: Merlin is a practicing wizard whose transformation magic (Wart as fish, squirrel, sparrow) and the wizards' duel with Madam Mim are among the most extensive in the classic Disney line; the sword in the stone is a real magical test of destiny; load-bearing, clears the strict gate easily. RELEVANCE: passes. SD=0: no societal decline; Uther's missing heir is a plot setup that Arthur's coronation fully resolves. LH=0: the sword is pulled, the prophecy is fulfilled, and Merlin returns to help; Arthur's self-doubt is a mild beat, not an unresolved loss. MC=0: nobody profits from wrongdoing and Mim is defeated; Ector's servant-like treatment of Wart is minor and ends in an apology. SC=0: no institution examined. RD=0: no one atones for real wrongdoing. NAI=0: nothing left unresolved. ED=1: G-rated, no deaths or graphic content; peril (pike, wolf, hawk, Mim's capture of Wart) is played comically, and Mim's dragon form comes in a gag-driven duel; below Sleeping Beauty's ED2 where the curse and dragon battle are treated seriously. Neighbor check: 1.725 is an exact 7-axis profile match with Final Fantasy I (ED1 only); Mary Poppins/Totoro/Kiki (1.5, all zeros) sit below and Sleeping Beauty (1.95, ED2) above. Boundary check: WIS 0.10 is far from the Tier 2 floor (0.222). Label check: "Very Bright Fantasy" fits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Miss Peregrine's Home for Peculiar Children</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ransom Riggs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENRE GATE: the peculiar children have real powers (invisibility, super strength, fire, levitation), Miss Peregrine is an ymbryne who becomes a bird and maintains a real time loop, and the wights and hollowgast are genuine supernatural predators; load-bearing, clears the strict gate easily. SCOPE: the 2011 novel only (book one); the 2016 Burton film diverges substantially (villain, year, deaths, ending) and is queued separately as item 96; sequels out of scope. RELEVANCE: passes. SD=1: the loop-bound world is fragile and the Holocaust backdrop (Abe's flight from Nazi Poland) gives it a sombre shadow, but the decay is mostly plot-driven by wights rather than a collapsing society; 2 considered and rejected. LH=2: Golan is defeated and Miss Peregrine is rescued, but the loop is destroyed, Miss Avocet is taken, Abe is dead, and the wights' threat remains. MC=1: wights exploit peculiars for gain, but virtue is not systematically punished. SC=0: no institution examined. RD=0: no antagonist atones and nothing turns on redemption. NAI=1: the persecution of peculiars is unresolved, but the posture at the end is determined flight rather than resignation; 2 considered. ED=3: hollowgast devour peculiars, mutilated sheep, several deaths, a gunshot, and creepy vintage-photo atmosphere with genuine detail; 4 ruled out as it is not the central element. Neighbor check: 3.8625 is an exact score tie with Shrek (3.86); closest similar profile Rise of the Guardians (3.525); Tier 3/4 boundary checked against NeverEnding Story, Twilight and Once Upon a Time (4.2), which carry heavier combinations. Label check: "Moderately Bright Fantasy" fits.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2334,7 +2343,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R167"/>
+  <dimension ref="A1:R168"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -11396,7 +11405,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="1" t="n">
         <v>1</v>
       </c>
@@ -11450,6 +11459,62 @@
       </c>
       <c r="R167" s="1" t="s">
         <v>499</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C168" s="1" t="s">
+        <v>500</v>
+      </c>
+      <c r="D168" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E168" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="F168" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G168" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H168" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I168" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="J168" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K168" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L168" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M168" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="N168" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O168" s="1" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="P168" s="1" t="n">
+        <v>3.8625</v>
+      </c>
+      <c r="Q168" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="R168" s="1" t="s">
+        <v>502</v>
       </c>
     </row>
   </sheetData>
@@ -11484,7 +11549,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11599,7 +11664,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add One Thousand and One Nights (Arabian Nights) to Tier 4
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1207" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1214" uniqueCount="508">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1531,6 +1531,15 @@
   </si>
   <si>
     <t xml:space="preserve">GENRE GATE: the peculiar children have real powers (invisibility, super strength, fire, levitation), Miss Peregrine is an ymbryne who becomes a bird and maintains a real time loop, and the wights and hollowgast are genuine supernatural predators; load-bearing, clears the strict gate easily. SCOPE: the 2011 novel only (book one); the 2016 Burton film diverges substantially (villain, year, deaths, ending) and is queued separately as item 96; sequels out of scope. RELEVANCE: passes. SD=1: the loop-bound world is fragile and the Holocaust backdrop (Abe's flight from Nazi Poland) gives it a sombre shadow, but the decay is mostly plot-driven by wights rather than a collapsing society; 2 considered and rejected. LH=2: Golan is defeated and Miss Peregrine is rescued, but the loop is destroyed, Miss Avocet is taken, Abe is dead, and the wights' threat remains. MC=1: wights exploit peculiars for gain, but virtue is not systematically punished. SC=0: no institution examined. RD=0: no antagonist atones and nothing turns on redemption. NAI=1: the persecution of peculiars is unresolved, but the posture at the end is determined flight rather than resignation; 2 considered. ED=3: hollowgast devour peculiars, mutilated sheep, several deaths, a gunshot, and creepy vintage-photo atmosphere with genuine detail; 4 ruled out as it is not the central element. Neighbor check: 3.8625 is an exact score tie with Shrek (3.86); closest similar profile Rise of the Guardians (3.525); Tier 3/4 boundary checked against NeverEnding Story, Twilight and Once Upon a Time (4.2), which carry heavier combinations. Label check: "Moderately Bright Fantasy" fits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One Thousand and One Nights (Arabian Nights)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traditional (Middle Eastern / Persian / Arabic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENRE GATE: jinn, ifrits, ghouls, the Roc, a flying ebony horse and magic objects recur across the collection and it is the root text of the Arabian fantasy tradition; clears the strict gate. SCOPE: the collection as traditionally received (Scheherazade frame, jinn tales, Sinbad, Galland-era additions Ali Baba and Aladdin); Disney's Aladdin stays separate; no single translation scored. RELEVANCE: passes; a share of the tales are historical or romantic with no magic, but the marvellous is the collection's identity. SD=1: the frame is a kingdom living under nightly executions, but the world of the tales is stable and the frame ends. LH=1: Scheherazade's wit ends the killing and Morgiana, Aladdin and Sinbad succeed, though many protagonists suffer under fate. MC=1: the providential frame usually punishes wickedness and rewards piety; cunning and betrayal pay off in many comic tales, so 2 considered. SC=2: the king's executions are state machinery (the vizier must supply a bride nightly) and caliphs and viziers act capriciously. RD=1: Shahryar's repentance takes 1,001 nights but costs him no punishment. NAI=2: the frame's murders are never answered and slavery, concubinage and women's subordination are treated as the natural order. ED=3: beheadings, a woman dismembered in a chest, cannibal ghouls, a spouse buried alive, and explicit sexual content (strongest in Burton and Mardrus); 4 ruled out as not the central element. Neighbor check: 4.875 is an exact 7-axis twin of The Shannara Chronicles; Pirates of the Caribbean, FMA: Brotherhood, Vox Machina and Ranking of Kings share the score via different profiles; Earthsea (4.65) sits below with far less violence and cynicism. Boundary check: Tier 5 cutoff is WIS 1.556, 0.056 away; MC=2 would give 5.2125 (tie with Tales from Earthsea). Label check: "Fantasy in Gray Tones" fits.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2343,7 +2352,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R168"/>
+  <dimension ref="A1:R169"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -11461,7 +11470,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="1" t="n">
         <v>3</v>
       </c>
@@ -11515,6 +11524,62 @@
       </c>
       <c r="R168" s="1" t="s">
         <v>502</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B169" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="D169" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E169" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="F169" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G169" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H169" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I169" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="J169" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K169" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="L169" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M169" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="N169" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="O169" s="1" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P169" s="1" t="n">
+        <v>4.875</v>
+      </c>
+      <c r="Q169" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="R169" s="1" t="s">
+        <v>505</v>
       </c>
     </row>
   </sheetData>
@@ -11549,7 +11614,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11664,7 +11729,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add The Princess and the Frog (2009) to Tier 2
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy_Grimdark_Scale_v2_WIP.xlsx
+++ b/Fantasy_Grimdark_Scale_v2_WIP.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1214" uniqueCount="508">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1221" uniqueCount="510">
   <si>
     <t xml:space="preserve">Fantasy Darkness Scale — Methodology v2</t>
   </si>
@@ -1540,6 +1540,12 @@
   </si>
   <si>
     <t xml:space="preserve">GENRE GATE: jinn, ifrits, ghouls, the Roc, a flying ebony horse and magic objects recur across the collection and it is the root text of the Arabian fantasy tradition; clears the strict gate. SCOPE: the collection as traditionally received (Scheherazade frame, jinn tales, Sinbad, Galland-era additions Ali Baba and Aladdin); Disney's Aladdin stays separate; no single translation scored. RELEVANCE: passes; a share of the tales are historical or romantic with no magic, but the marvellous is the collection's identity. SD=1: the frame is a kingdom living under nightly executions, but the world of the tales is stable and the frame ends. LH=1: Scheherazade's wit ends the killing and Morgiana, Aladdin and Sinbad succeed, though many protagonists suffer under fate. MC=1: the providential frame usually punishes wickedness and rewards piety; cunning and betrayal pay off in many comic tales, so 2 considered. SC=2: the king's executions are state machinery (the vizier must supply a bride nightly) and caliphs and viziers act capriciously. RD=1: Shahryar's repentance takes 1,001 nights but costs him no punishment. NAI=2: the frame's murders are never answered and slavery, concubinage and women's subordination are treated as the natural order. ED=3: beheadings, a woman dismembered in a chest, cannibal ghouls, a spouse buried alive, and explicit sexual content (strongest in Burton and Mardrus); 4 ruled out as not the central element. Neighbor check: 4.875 is an exact 7-axis twin of The Shannara Chronicles; Pirates of the Caribbean, FMA: Brotherhood, Vox Machina and Ranking of Kings share the score via different profiles; Earthsea (4.65) sits below with far less violence and cynicism. Boundary check: Tier 5 cutoff is WIS 1.556, 0.056 away; MC=2 would give 5.2125 (tie with Tales from Earthsea). Label check: "Fantasy in Gray Tones" fits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Princess and the Frog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GENRE GATE: Dr. Facilier is a voodoo sorcerer with a blood-bound talisman and 'Friends on the Other Side' who supply shadow demons; the frog curse and Mama Odie's fairy-godmother role drive the whole plot; clears the strict gate easily. SCOPE: the 2009 film only; the E. D. Baker novel and the Grimm tale are separate sources. RELEVANCE: passes. SD=0: Facilier's plan to take the city's souls fails completely and nothing else in the world is decaying. LH=0: Tiana destroys the talisman and Facilier is dragged to the underworld; Ray's death is mourned, then he is transfigured into a star. MC=1: Facilier's plot nearly succeeds (Lawrence passes as Naveen and almost marries Charlotte), but Tiana's hard work and honesty are rewarded. SC=0: no institution is examined; the Fenner brothers' condescension is a personal obstacle (critics note the film sanitizes Jim Crow, but the score reflects what the work shows; 1 considered). RD=1: Naveen must give up his easy-money plan and learn to work, and Tiana refuses Facilier's offer of her dream restaurant. NAI=0: Facilier is destroyed, Lawrence arrested, nothing left open. ED=2: the shadow-demon sequences are among Disney's scarier ones, Ray dies on screen, and frog hunters fire guns at the leads; G-rated with no gore; 3 considered. Neighbor check: 2.625 is an exact 7-axis twin of Enchanted; shares the score with The Wizard of Oz, Alice in Wonderland (2010-2016), Onward and The Sorcerer's Apprentice via different profiles; Aladdin (2.96) sits above with extra corruption and injustice; Tangled (3.19) above with ED3 and RD2; Cinderella (2.29) below. Boundary check: WIS 0.50 vs Tier 3 floor 0.667; ED3 would give 2.85, still Tier 2. Label check: "Bright Fantasy" fits.</t>
   </si>
   <si>
     <t xml:space="preserve">Works scored (v2 WIP)</t>
@@ -2352,7 +2358,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R169"/>
+  <dimension ref="A1:R170"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -11526,7 +11532,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="1" t="n">
         <v>4</v>
       </c>
@@ -11580,6 +11586,62 @@
       </c>
       <c r="R169" s="1" t="s">
         <v>505</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="D170" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E170" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F170" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G170" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H170" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I170" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J170" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K170" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L170" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M170" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N170" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="O170" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P170" s="1" t="n">
+        <v>2.625</v>
+      </c>
+      <c r="Q170" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="R170" s="1" t="s">
+        <v>507</v>
       </c>
     </row>
   </sheetData>
@@ -11614,7 +11676,7 @@
         <v>91</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11729,7 +11791,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
   </sheetData>

</xml_diff>